<commit_message>
Complete Receipt-X v2 foundation and UI improvements
</commit_message>
<xml_diff>
--- a/PRODUCT_MASTER/RECEIPT-X_PRODUCT_MASTER.xlsx
+++ b/PRODUCT_MASTER/RECEIPT-X_PRODUCT_MASTER.xlsx
@@ -9,10 +9,24 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8180"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8180" firstSheet="9" activeTab="14"/>
   </bookViews>
   <sheets>
     <sheet name="PWANI OIL PRODUCTS" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="7" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="8" r:id="rId3"/>
+    <sheet name="Sheet4" sheetId="9" r:id="rId4"/>
+    <sheet name="Sheet5" sheetId="10" r:id="rId5"/>
+    <sheet name="Sheet6" sheetId="11" r:id="rId6"/>
+    <sheet name="Sheet7" sheetId="12" r:id="rId7"/>
+    <sheet name="Sheet8" sheetId="13" r:id="rId8"/>
+    <sheet name="VIPINGO INDUSTRIES" sheetId="2" r:id="rId9"/>
+    <sheet name="MVITA OIL" sheetId="3" r:id="rId10"/>
+    <sheet name="YEMKEN" sheetId="4" r:id="rId11"/>
+    <sheet name="KILIMANJARO BISCUITS" sheetId="5" r:id="rId12"/>
+    <sheet name="KENAFRIC" sheetId="6" r:id="rId13"/>
+    <sheet name="MZURI SWEETS" sheetId="14" r:id="rId14"/>
+    <sheet name="AZAM" sheetId="15" r:id="rId15"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -24,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="48">
   <si>
     <t>Brand</t>
   </si>
@@ -102,6 +116,72 @@
   </si>
   <si>
     <t>PRICE</t>
+  </si>
+  <si>
+    <t>Golden Drop</t>
+  </si>
+  <si>
+    <t>Goden Drop</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Golden Drop</t>
+  </si>
+  <si>
+    <t>Cookstar Yellow</t>
+  </si>
+  <si>
+    <t>5kg</t>
+  </si>
+  <si>
+    <t>10kg</t>
+  </si>
+  <si>
+    <t>17kg</t>
+  </si>
+  <si>
+    <t>Karaih</t>
+  </si>
+  <si>
+    <t>Mfalme</t>
+  </si>
+  <si>
+    <t>Redsun</t>
+  </si>
+  <si>
+    <t>5og</t>
+  </si>
+  <si>
+    <t>Redsun 400g</t>
+  </si>
+  <si>
+    <t>400g</t>
+  </si>
+  <si>
+    <t>Parle G</t>
+  </si>
+  <si>
+    <t>74x4g</t>
+  </si>
+  <si>
+    <t>300pcs</t>
+  </si>
+  <si>
+    <t>Brittania</t>
+  </si>
+  <si>
+    <t>72x4g</t>
+  </si>
+  <si>
+    <t>Mr Berry</t>
+  </si>
+  <si>
+    <t>20x50pcs</t>
+  </si>
+  <si>
+    <t>Azam Energy Drink</t>
+  </si>
+  <si>
+    <t>300ml</t>
   </si>
 </sst>
 </file>
@@ -893,4 +973,561 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="16.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>